<commit_message>
Enhance coach response review rubric
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/coach_response_review_workbook_fair_mini_study_20_20260511.zh.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/coach_response_review_workbook_fair_mini_study_20_20260511.zh.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'盲评表'!$A$2:$R$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'盲评表'!$A$2:$W$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -261,20 +261,45 @@
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>如果回复使用小例子，例子是否引导学生提炼可迁移的桥梁关系，而不是只完成一次临时任务。没有小例子但回复合理时可评 2。</t>
+        <t>如果回复使用或应该使用小例子，例子是否引导学生提炼可迁移的桥梁关系，而不是只完成一次临时任务。不适用时先在“微型例子是否适用”选 N/A。</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
+        <t>判断这条回复是否需要单独评价微型例子。若回复没有使用例子且本轮不需要例子，选 N/A，微型例子分数可留空。</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
         <t>判断这条回复实际有没有泄露当前关键桥或完整答案/代码。</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>同一个样本如果有多条匿名回复，可按质量排序。1 表示最好，可留空。</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>整体看，你作为教练愿不愿意把这条回复给学生看。1=很差，5=优秀。</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>把细项放到一边，判断这条回复是否可以直接给学生看。</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>你对本次评分的把握程度。低置信样本后续应进入讨论或双标。</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>是否需要二次讨论或裁决。适合边界样本、信息不足或多个系统难分高下的情况。</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>评完后选“已评完”；不确定就选“需要讨论”。</t>
       </text>
@@ -572,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -619,7 +644,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>六个维度都用 0/1/2：2=好，1=一般，0=差。每格都有中文下拉解释。</t>
+          <t>细维度用 0/1/2：2=好，1=一般，0=差；总体质量用 1/2/3/4/5。每格都有中文下拉解释。</t>
         </is>
       </c>
     </row>
@@ -638,10 +663,34 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>微型例子</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>先判断这条回复是否需要评价微型例子；不适用时选 N/A/不适用，微型例子分数可留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>整体判断</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>总体质量和“是否愿意给学生看”用于保留你的教练直觉，不替代细项评分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>不确定怎么办</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>review_status 选“不确定，需要讨论”，备注写原因。</t>
         </is>
@@ -658,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R142"/>
+  <dimension ref="A1:W142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -675,10 +724,15 @@
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -754,20 +808,45 @@
       </c>
       <c r="O1" s="4" t="inlineStr">
         <is>
+          <t>微型例子是否适用</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
           <t>泄露标签</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>同题回复排序</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>总体质量 1-5</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>是否愿意给学生看</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>评分置信度</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>是否需要讨论</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>评审状态</t>
         </is>
@@ -846,20 +925,45 @@
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
+          <t>coach_micro_example_applicability</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
           <t>coach_leakage_label</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>coach_preference_rank</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>coach_overall_quality_score</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>coach_would_show_to_student</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>coach_reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>coach_needs_discussion</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>coach_notes</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>review_status</t>
         </is>
@@ -914,7 +1018,12 @@
       <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr"/>
       <c r="Q3" s="7" t="inlineStr"/>
-      <c r="R3" s="7" t="inlineStr">
+      <c r="R3" s="7" t="inlineStr"/>
+      <c r="S3" s="7" t="inlineStr"/>
+      <c r="T3" s="7" t="inlineStr"/>
+      <c r="U3" s="7" t="inlineStr"/>
+      <c r="V3" s="7" t="inlineStr"/>
+      <c r="W3" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -962,7 +1071,12 @@
       <c r="O4" s="7" t="inlineStr"/>
       <c r="P4" s="7" t="inlineStr"/>
       <c r="Q4" s="7" t="inlineStr"/>
-      <c r="R4" s="7" t="inlineStr">
+      <c r="R4" s="7" t="inlineStr"/>
+      <c r="S4" s="7" t="inlineStr"/>
+      <c r="T4" s="7" t="inlineStr"/>
+      <c r="U4" s="7" t="inlineStr"/>
+      <c r="V4" s="7" t="inlineStr"/>
+      <c r="W4" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1012,7 +1126,12 @@
       <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="7" t="inlineStr"/>
       <c r="Q5" s="7" t="inlineStr"/>
-      <c r="R5" s="7" t="inlineStr">
+      <c r="R5" s="7" t="inlineStr"/>
+      <c r="S5" s="7" t="inlineStr"/>
+      <c r="T5" s="7" t="inlineStr"/>
+      <c r="U5" s="7" t="inlineStr"/>
+      <c r="V5" s="7" t="inlineStr"/>
+      <c r="W5" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1071,7 +1190,12 @@
       <c r="O6" s="7" t="inlineStr"/>
       <c r="P6" s="7" t="inlineStr"/>
       <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr">
+      <c r="R6" s="7" t="inlineStr"/>
+      <c r="S6" s="7" t="inlineStr"/>
+      <c r="T6" s="7" t="inlineStr"/>
+      <c r="U6" s="7" t="inlineStr"/>
+      <c r="V6" s="7" t="inlineStr"/>
+      <c r="W6" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1119,7 +1243,12 @@
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr"/>
       <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr">
+      <c r="R7" s="7" t="inlineStr"/>
+      <c r="S7" s="7" t="inlineStr"/>
+      <c r="T7" s="7" t="inlineStr"/>
+      <c r="U7" s="7" t="inlineStr"/>
+      <c r="V7" s="7" t="inlineStr"/>
+      <c r="W7" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1177,7 +1306,12 @@
       <c r="O8" s="7" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr"/>
       <c r="Q8" s="7" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr">
+      <c r="R8" s="7" t="inlineStr"/>
+      <c r="S8" s="7" t="inlineStr"/>
+      <c r="T8" s="7" t="inlineStr"/>
+      <c r="U8" s="7" t="inlineStr"/>
+      <c r="V8" s="7" t="inlineStr"/>
+      <c r="W8" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1232,7 +1366,12 @@
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr"/>
       <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr">
+      <c r="R9" s="7" t="inlineStr"/>
+      <c r="S9" s="7" t="inlineStr"/>
+      <c r="T9" s="7" t="inlineStr"/>
+      <c r="U9" s="7" t="inlineStr"/>
+      <c r="V9" s="7" t="inlineStr"/>
+      <c r="W9" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1280,7 +1419,12 @@
       <c r="O10" s="7" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr"/>
       <c r="Q10" s="7" t="inlineStr"/>
-      <c r="R10" s="7" t="inlineStr">
+      <c r="R10" s="7" t="inlineStr"/>
+      <c r="S10" s="7" t="inlineStr"/>
+      <c r="T10" s="7" t="inlineStr"/>
+      <c r="U10" s="7" t="inlineStr"/>
+      <c r="V10" s="7" t="inlineStr"/>
+      <c r="W10" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1337,7 +1481,12 @@
       <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr"/>
       <c r="Q11" s="7" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr">
+      <c r="R11" s="7" t="inlineStr"/>
+      <c r="S11" s="7" t="inlineStr"/>
+      <c r="T11" s="7" t="inlineStr"/>
+      <c r="U11" s="7" t="inlineStr"/>
+      <c r="V11" s="7" t="inlineStr"/>
+      <c r="W11" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1390,7 +1539,12 @@
       <c r="O12" s="7" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr"/>
       <c r="Q12" s="7" t="inlineStr"/>
-      <c r="R12" s="7" t="inlineStr">
+      <c r="R12" s="7" t="inlineStr"/>
+      <c r="S12" s="7" t="inlineStr"/>
+      <c r="T12" s="7" t="inlineStr"/>
+      <c r="U12" s="7" t="inlineStr"/>
+      <c r="V12" s="7" t="inlineStr"/>
+      <c r="W12" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1438,7 +1592,12 @@
       <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr"/>
       <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr">
+      <c r="R13" s="7" t="inlineStr"/>
+      <c r="S13" s="7" t="inlineStr"/>
+      <c r="T13" s="7" t="inlineStr"/>
+      <c r="U13" s="7" t="inlineStr"/>
+      <c r="V13" s="7" t="inlineStr"/>
+      <c r="W13" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1486,7 +1645,12 @@
       <c r="O14" s="7" t="inlineStr"/>
       <c r="P14" s="7" t="inlineStr"/>
       <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr">
+      <c r="R14" s="7" t="inlineStr"/>
+      <c r="S14" s="7" t="inlineStr"/>
+      <c r="T14" s="7" t="inlineStr"/>
+      <c r="U14" s="7" t="inlineStr"/>
+      <c r="V14" s="7" t="inlineStr"/>
+      <c r="W14" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1542,7 +1706,12 @@
       <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr"/>
       <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr">
+      <c r="R15" s="7" t="inlineStr"/>
+      <c r="S15" s="7" t="inlineStr"/>
+      <c r="T15" s="7" t="inlineStr"/>
+      <c r="U15" s="7" t="inlineStr"/>
+      <c r="V15" s="7" t="inlineStr"/>
+      <c r="W15" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1599,7 +1768,12 @@
       <c r="O16" s="7" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr"/>
       <c r="Q16" s="7" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr">
+      <c r="R16" s="7" t="inlineStr"/>
+      <c r="S16" s="7" t="inlineStr"/>
+      <c r="T16" s="7" t="inlineStr"/>
+      <c r="U16" s="7" t="inlineStr"/>
+      <c r="V16" s="7" t="inlineStr"/>
+      <c r="W16" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1669,7 +1843,12 @@
       <c r="O17" s="7" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr"/>
       <c r="Q17" s="7" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr">
+      <c r="R17" s="7" t="inlineStr"/>
+      <c r="S17" s="7" t="inlineStr"/>
+      <c r="T17" s="7" t="inlineStr"/>
+      <c r="U17" s="7" t="inlineStr"/>
+      <c r="V17" s="7" t="inlineStr"/>
+      <c r="W17" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1717,7 +1896,12 @@
       <c r="O18" s="7" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr"/>
       <c r="Q18" s="7" t="inlineStr"/>
-      <c r="R18" s="7" t="inlineStr">
+      <c r="R18" s="7" t="inlineStr"/>
+      <c r="S18" s="7" t="inlineStr"/>
+      <c r="T18" s="7" t="inlineStr"/>
+      <c r="U18" s="7" t="inlineStr"/>
+      <c r="V18" s="7" t="inlineStr"/>
+      <c r="W18" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1776,7 +1960,12 @@
       <c r="O19" s="7" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr"/>
       <c r="Q19" s="7" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr">
+      <c r="R19" s="7" t="inlineStr"/>
+      <c r="S19" s="7" t="inlineStr"/>
+      <c r="T19" s="7" t="inlineStr"/>
+      <c r="U19" s="7" t="inlineStr"/>
+      <c r="V19" s="7" t="inlineStr"/>
+      <c r="W19" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1828,7 +2017,12 @@
       <c r="O20" s="7" t="inlineStr"/>
       <c r="P20" s="7" t="inlineStr"/>
       <c r="Q20" s="7" t="inlineStr"/>
-      <c r="R20" s="7" t="inlineStr">
+      <c r="R20" s="7" t="inlineStr"/>
+      <c r="S20" s="7" t="inlineStr"/>
+      <c r="T20" s="7" t="inlineStr"/>
+      <c r="U20" s="7" t="inlineStr"/>
+      <c r="V20" s="7" t="inlineStr"/>
+      <c r="W20" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1878,7 +2072,12 @@
       <c r="O21" s="7" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr"/>
       <c r="Q21" s="7" t="inlineStr"/>
-      <c r="R21" s="7" t="inlineStr">
+      <c r="R21" s="7" t="inlineStr"/>
+      <c r="S21" s="7" t="inlineStr"/>
+      <c r="T21" s="7" t="inlineStr"/>
+      <c r="U21" s="7" t="inlineStr"/>
+      <c r="V21" s="7" t="inlineStr"/>
+      <c r="W21" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1934,7 +2133,12 @@
       <c r="O22" s="7" t="inlineStr"/>
       <c r="P22" s="7" t="inlineStr"/>
       <c r="Q22" s="7" t="inlineStr"/>
-      <c r="R22" s="7" t="inlineStr">
+      <c r="R22" s="7" t="inlineStr"/>
+      <c r="S22" s="7" t="inlineStr"/>
+      <c r="T22" s="7" t="inlineStr"/>
+      <c r="U22" s="7" t="inlineStr"/>
+      <c r="V22" s="7" t="inlineStr"/>
+      <c r="W22" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -1987,7 +2191,12 @@
       <c r="O23" s="7" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr"/>
       <c r="Q23" s="7" t="inlineStr"/>
-      <c r="R23" s="7" t="inlineStr">
+      <c r="R23" s="7" t="inlineStr"/>
+      <c r="S23" s="7" t="inlineStr"/>
+      <c r="T23" s="7" t="inlineStr"/>
+      <c r="U23" s="7" t="inlineStr"/>
+      <c r="V23" s="7" t="inlineStr"/>
+      <c r="W23" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2045,7 +2254,12 @@
       <c r="O24" s="7" t="inlineStr"/>
       <c r="P24" s="7" t="inlineStr"/>
       <c r="Q24" s="7" t="inlineStr"/>
-      <c r="R24" s="7" t="inlineStr">
+      <c r="R24" s="7" t="inlineStr"/>
+      <c r="S24" s="7" t="inlineStr"/>
+      <c r="T24" s="7" t="inlineStr"/>
+      <c r="U24" s="7" t="inlineStr"/>
+      <c r="V24" s="7" t="inlineStr"/>
+      <c r="W24" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2095,7 +2309,12 @@
       <c r="O25" s="7" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr"/>
       <c r="Q25" s="7" t="inlineStr"/>
-      <c r="R25" s="7" t="inlineStr">
+      <c r="R25" s="7" t="inlineStr"/>
+      <c r="S25" s="7" t="inlineStr"/>
+      <c r="T25" s="7" t="inlineStr"/>
+      <c r="U25" s="7" t="inlineStr"/>
+      <c r="V25" s="7" t="inlineStr"/>
+      <c r="W25" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2151,7 +2370,12 @@
       <c r="O26" s="7" t="inlineStr"/>
       <c r="P26" s="7" t="inlineStr"/>
       <c r="Q26" s="7" t="inlineStr"/>
-      <c r="R26" s="7" t="inlineStr">
+      <c r="R26" s="7" t="inlineStr"/>
+      <c r="S26" s="7" t="inlineStr"/>
+      <c r="T26" s="7" t="inlineStr"/>
+      <c r="U26" s="7" t="inlineStr"/>
+      <c r="V26" s="7" t="inlineStr"/>
+      <c r="W26" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2206,7 +2430,12 @@
       <c r="O27" s="7" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr"/>
       <c r="Q27" s="7" t="inlineStr"/>
-      <c r="R27" s="7" t="inlineStr">
+      <c r="R27" s="7" t="inlineStr"/>
+      <c r="S27" s="7" t="inlineStr"/>
+      <c r="T27" s="7" t="inlineStr"/>
+      <c r="U27" s="7" t="inlineStr"/>
+      <c r="V27" s="7" t="inlineStr"/>
+      <c r="W27" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2266,7 +2495,12 @@
       <c r="O28" s="7" t="inlineStr"/>
       <c r="P28" s="7" t="inlineStr"/>
       <c r="Q28" s="7" t="inlineStr"/>
-      <c r="R28" s="7" t="inlineStr">
+      <c r="R28" s="7" t="inlineStr"/>
+      <c r="S28" s="7" t="inlineStr"/>
+      <c r="T28" s="7" t="inlineStr"/>
+      <c r="U28" s="7" t="inlineStr"/>
+      <c r="V28" s="7" t="inlineStr"/>
+      <c r="W28" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2335,7 +2569,12 @@
       <c r="O29" s="7" t="inlineStr"/>
       <c r="P29" s="7" t="inlineStr"/>
       <c r="Q29" s="7" t="inlineStr"/>
-      <c r="R29" s="7" t="inlineStr">
+      <c r="R29" s="7" t="inlineStr"/>
+      <c r="S29" s="7" t="inlineStr"/>
+      <c r="T29" s="7" t="inlineStr"/>
+      <c r="U29" s="7" t="inlineStr"/>
+      <c r="V29" s="7" t="inlineStr"/>
+      <c r="W29" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2388,7 +2627,12 @@
       <c r="O30" s="7" t="inlineStr"/>
       <c r="P30" s="7" t="inlineStr"/>
       <c r="Q30" s="7" t="inlineStr"/>
-      <c r="R30" s="7" t="inlineStr">
+      <c r="R30" s="7" t="inlineStr"/>
+      <c r="S30" s="7" t="inlineStr"/>
+      <c r="T30" s="7" t="inlineStr"/>
+      <c r="U30" s="7" t="inlineStr"/>
+      <c r="V30" s="7" t="inlineStr"/>
+      <c r="W30" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2444,7 +2688,12 @@
       <c r="O31" s="7" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr"/>
       <c r="Q31" s="7" t="inlineStr"/>
-      <c r="R31" s="7" t="inlineStr">
+      <c r="R31" s="7" t="inlineStr"/>
+      <c r="S31" s="7" t="inlineStr"/>
+      <c r="T31" s="7" t="inlineStr"/>
+      <c r="U31" s="7" t="inlineStr"/>
+      <c r="V31" s="7" t="inlineStr"/>
+      <c r="W31" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2497,7 +2746,12 @@
       <c r="O32" s="7" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr"/>
       <c r="Q32" s="7" t="inlineStr"/>
-      <c r="R32" s="7" t="inlineStr">
+      <c r="R32" s="7" t="inlineStr"/>
+      <c r="S32" s="7" t="inlineStr"/>
+      <c r="T32" s="7" t="inlineStr"/>
+      <c r="U32" s="7" t="inlineStr"/>
+      <c r="V32" s="7" t="inlineStr"/>
+      <c r="W32" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2555,7 +2809,12 @@
       <c r="O33" s="7" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr"/>
       <c r="Q33" s="7" t="inlineStr"/>
-      <c r="R33" s="7" t="inlineStr">
+      <c r="R33" s="7" t="inlineStr"/>
+      <c r="S33" s="7" t="inlineStr"/>
+      <c r="T33" s="7" t="inlineStr"/>
+      <c r="U33" s="7" t="inlineStr"/>
+      <c r="V33" s="7" t="inlineStr"/>
+      <c r="W33" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2615,7 +2874,12 @@
       <c r="O34" s="7" t="inlineStr"/>
       <c r="P34" s="7" t="inlineStr"/>
       <c r="Q34" s="7" t="inlineStr"/>
-      <c r="R34" s="7" t="inlineStr">
+      <c r="R34" s="7" t="inlineStr"/>
+      <c r="S34" s="7" t="inlineStr"/>
+      <c r="T34" s="7" t="inlineStr"/>
+      <c r="U34" s="7" t="inlineStr"/>
+      <c r="V34" s="7" t="inlineStr"/>
+      <c r="W34" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2674,7 +2938,12 @@
       <c r="O35" s="7" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr"/>
       <c r="Q35" s="7" t="inlineStr"/>
-      <c r="R35" s="7" t="inlineStr">
+      <c r="R35" s="7" t="inlineStr"/>
+      <c r="S35" s="7" t="inlineStr"/>
+      <c r="T35" s="7" t="inlineStr"/>
+      <c r="U35" s="7" t="inlineStr"/>
+      <c r="V35" s="7" t="inlineStr"/>
+      <c r="W35" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2722,7 +2991,12 @@
       <c r="O36" s="7" t="inlineStr"/>
       <c r="P36" s="7" t="inlineStr"/>
       <c r="Q36" s="7" t="inlineStr"/>
-      <c r="R36" s="7" t="inlineStr">
+      <c r="R36" s="7" t="inlineStr"/>
+      <c r="S36" s="7" t="inlineStr"/>
+      <c r="T36" s="7" t="inlineStr"/>
+      <c r="U36" s="7" t="inlineStr"/>
+      <c r="V36" s="7" t="inlineStr"/>
+      <c r="W36" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2773,7 +3047,12 @@
       <c r="O37" s="7" t="inlineStr"/>
       <c r="P37" s="7" t="inlineStr"/>
       <c r="Q37" s="7" t="inlineStr"/>
-      <c r="R37" s="7" t="inlineStr">
+      <c r="R37" s="7" t="inlineStr"/>
+      <c r="S37" s="7" t="inlineStr"/>
+      <c r="T37" s="7" t="inlineStr"/>
+      <c r="U37" s="7" t="inlineStr"/>
+      <c r="V37" s="7" t="inlineStr"/>
+      <c r="W37" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2821,7 +3100,12 @@
       <c r="O38" s="7" t="inlineStr"/>
       <c r="P38" s="7" t="inlineStr"/>
       <c r="Q38" s="7" t="inlineStr"/>
-      <c r="R38" s="7" t="inlineStr">
+      <c r="R38" s="7" t="inlineStr"/>
+      <c r="S38" s="7" t="inlineStr"/>
+      <c r="T38" s="7" t="inlineStr"/>
+      <c r="U38" s="7" t="inlineStr"/>
+      <c r="V38" s="7" t="inlineStr"/>
+      <c r="W38" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2871,7 +3155,12 @@
       <c r="O39" s="7" t="inlineStr"/>
       <c r="P39" s="7" t="inlineStr"/>
       <c r="Q39" s="7" t="inlineStr"/>
-      <c r="R39" s="7" t="inlineStr">
+      <c r="R39" s="7" t="inlineStr"/>
+      <c r="S39" s="7" t="inlineStr"/>
+      <c r="T39" s="7" t="inlineStr"/>
+      <c r="U39" s="7" t="inlineStr"/>
+      <c r="V39" s="7" t="inlineStr"/>
+      <c r="W39" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2919,7 +3208,12 @@
       <c r="O40" s="7" t="inlineStr"/>
       <c r="P40" s="7" t="inlineStr"/>
       <c r="Q40" s="7" t="inlineStr"/>
-      <c r="R40" s="7" t="inlineStr">
+      <c r="R40" s="7" t="inlineStr"/>
+      <c r="S40" s="7" t="inlineStr"/>
+      <c r="T40" s="7" t="inlineStr"/>
+      <c r="U40" s="7" t="inlineStr"/>
+      <c r="V40" s="7" t="inlineStr"/>
+      <c r="W40" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -2971,7 +3265,12 @@
       <c r="O41" s="7" t="inlineStr"/>
       <c r="P41" s="7" t="inlineStr"/>
       <c r="Q41" s="7" t="inlineStr"/>
-      <c r="R41" s="7" t="inlineStr">
+      <c r="R41" s="7" t="inlineStr"/>
+      <c r="S41" s="7" t="inlineStr"/>
+      <c r="T41" s="7" t="inlineStr"/>
+      <c r="U41" s="7" t="inlineStr"/>
+      <c r="V41" s="7" t="inlineStr"/>
+      <c r="W41" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3024,7 +3323,12 @@
       <c r="O42" s="7" t="inlineStr"/>
       <c r="P42" s="7" t="inlineStr"/>
       <c r="Q42" s="7" t="inlineStr"/>
-      <c r="R42" s="7" t="inlineStr">
+      <c r="R42" s="7" t="inlineStr"/>
+      <c r="S42" s="7" t="inlineStr"/>
+      <c r="T42" s="7" t="inlineStr"/>
+      <c r="U42" s="7" t="inlineStr"/>
+      <c r="V42" s="7" t="inlineStr"/>
+      <c r="W42" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3076,7 +3380,12 @@
       <c r="O43" s="7" t="inlineStr"/>
       <c r="P43" s="7" t="inlineStr"/>
       <c r="Q43" s="7" t="inlineStr"/>
-      <c r="R43" s="7" t="inlineStr">
+      <c r="R43" s="7" t="inlineStr"/>
+      <c r="S43" s="7" t="inlineStr"/>
+      <c r="T43" s="7" t="inlineStr"/>
+      <c r="U43" s="7" t="inlineStr"/>
+      <c r="V43" s="7" t="inlineStr"/>
+      <c r="W43" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3130,7 +3439,12 @@
       <c r="O44" s="7" t="inlineStr"/>
       <c r="P44" s="7" t="inlineStr"/>
       <c r="Q44" s="7" t="inlineStr"/>
-      <c r="R44" s="7" t="inlineStr">
+      <c r="R44" s="7" t="inlineStr"/>
+      <c r="S44" s="7" t="inlineStr"/>
+      <c r="T44" s="7" t="inlineStr"/>
+      <c r="U44" s="7" t="inlineStr"/>
+      <c r="V44" s="7" t="inlineStr"/>
+      <c r="W44" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3182,7 +3496,12 @@
       <c r="O45" s="7" t="inlineStr"/>
       <c r="P45" s="7" t="inlineStr"/>
       <c r="Q45" s="7" t="inlineStr"/>
-      <c r="R45" s="7" t="inlineStr">
+      <c r="R45" s="7" t="inlineStr"/>
+      <c r="S45" s="7" t="inlineStr"/>
+      <c r="T45" s="7" t="inlineStr"/>
+      <c r="U45" s="7" t="inlineStr"/>
+      <c r="V45" s="7" t="inlineStr"/>
+      <c r="W45" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3236,7 +3555,12 @@
       <c r="O46" s="7" t="inlineStr"/>
       <c r="P46" s="7" t="inlineStr"/>
       <c r="Q46" s="7" t="inlineStr"/>
-      <c r="R46" s="7" t="inlineStr">
+      <c r="R46" s="7" t="inlineStr"/>
+      <c r="S46" s="7" t="inlineStr"/>
+      <c r="T46" s="7" t="inlineStr"/>
+      <c r="U46" s="7" t="inlineStr"/>
+      <c r="V46" s="7" t="inlineStr"/>
+      <c r="W46" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3287,7 +3611,12 @@
       <c r="O47" s="7" t="inlineStr"/>
       <c r="P47" s="7" t="inlineStr"/>
       <c r="Q47" s="7" t="inlineStr"/>
-      <c r="R47" s="7" t="inlineStr">
+      <c r="R47" s="7" t="inlineStr"/>
+      <c r="S47" s="7" t="inlineStr"/>
+      <c r="T47" s="7" t="inlineStr"/>
+      <c r="U47" s="7" t="inlineStr"/>
+      <c r="V47" s="7" t="inlineStr"/>
+      <c r="W47" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3345,7 +3674,12 @@
       <c r="O48" s="7" t="inlineStr"/>
       <c r="P48" s="7" t="inlineStr"/>
       <c r="Q48" s="7" t="inlineStr"/>
-      <c r="R48" s="7" t="inlineStr">
+      <c r="R48" s="7" t="inlineStr"/>
+      <c r="S48" s="7" t="inlineStr"/>
+      <c r="T48" s="7" t="inlineStr"/>
+      <c r="U48" s="7" t="inlineStr"/>
+      <c r="V48" s="7" t="inlineStr"/>
+      <c r="W48" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3405,7 +3739,12 @@
       <c r="O49" s="7" t="inlineStr"/>
       <c r="P49" s="7" t="inlineStr"/>
       <c r="Q49" s="7" t="inlineStr"/>
-      <c r="R49" s="7" t="inlineStr">
+      <c r="R49" s="7" t="inlineStr"/>
+      <c r="S49" s="7" t="inlineStr"/>
+      <c r="T49" s="7" t="inlineStr"/>
+      <c r="U49" s="7" t="inlineStr"/>
+      <c r="V49" s="7" t="inlineStr"/>
+      <c r="W49" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3464,7 +3803,12 @@
       <c r="O50" s="7" t="inlineStr"/>
       <c r="P50" s="7" t="inlineStr"/>
       <c r="Q50" s="7" t="inlineStr"/>
-      <c r="R50" s="7" t="inlineStr">
+      <c r="R50" s="7" t="inlineStr"/>
+      <c r="S50" s="7" t="inlineStr"/>
+      <c r="T50" s="7" t="inlineStr"/>
+      <c r="U50" s="7" t="inlineStr"/>
+      <c r="V50" s="7" t="inlineStr"/>
+      <c r="W50" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3513,7 +3857,12 @@
       <c r="O51" s="7" t="inlineStr"/>
       <c r="P51" s="7" t="inlineStr"/>
       <c r="Q51" s="7" t="inlineStr"/>
-      <c r="R51" s="7" t="inlineStr">
+      <c r="R51" s="7" t="inlineStr"/>
+      <c r="S51" s="7" t="inlineStr"/>
+      <c r="T51" s="7" t="inlineStr"/>
+      <c r="U51" s="7" t="inlineStr"/>
+      <c r="V51" s="7" t="inlineStr"/>
+      <c r="W51" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3562,7 +3911,12 @@
       <c r="O52" s="7" t="inlineStr"/>
       <c r="P52" s="7" t="inlineStr"/>
       <c r="Q52" s="7" t="inlineStr"/>
-      <c r="R52" s="7" t="inlineStr">
+      <c r="R52" s="7" t="inlineStr"/>
+      <c r="S52" s="7" t="inlineStr"/>
+      <c r="T52" s="7" t="inlineStr"/>
+      <c r="U52" s="7" t="inlineStr"/>
+      <c r="V52" s="7" t="inlineStr"/>
+      <c r="W52" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3612,7 +3966,12 @@
       <c r="O53" s="7" t="inlineStr"/>
       <c r="P53" s="7" t="inlineStr"/>
       <c r="Q53" s="7" t="inlineStr"/>
-      <c r="R53" s="7" t="inlineStr">
+      <c r="R53" s="7" t="inlineStr"/>
+      <c r="S53" s="7" t="inlineStr"/>
+      <c r="T53" s="7" t="inlineStr"/>
+      <c r="U53" s="7" t="inlineStr"/>
+      <c r="V53" s="7" t="inlineStr"/>
+      <c r="W53" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3678,7 +4037,12 @@
       <c r="O54" s="7" t="inlineStr"/>
       <c r="P54" s="7" t="inlineStr"/>
       <c r="Q54" s="7" t="inlineStr"/>
-      <c r="R54" s="7" t="inlineStr">
+      <c r="R54" s="7" t="inlineStr"/>
+      <c r="S54" s="7" t="inlineStr"/>
+      <c r="T54" s="7" t="inlineStr"/>
+      <c r="U54" s="7" t="inlineStr"/>
+      <c r="V54" s="7" t="inlineStr"/>
+      <c r="W54" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3746,7 +4110,12 @@
       <c r="O55" s="7" t="inlineStr"/>
       <c r="P55" s="7" t="inlineStr"/>
       <c r="Q55" s="7" t="inlineStr"/>
-      <c r="R55" s="7" t="inlineStr">
+      <c r="R55" s="7" t="inlineStr"/>
+      <c r="S55" s="7" t="inlineStr"/>
+      <c r="T55" s="7" t="inlineStr"/>
+      <c r="U55" s="7" t="inlineStr"/>
+      <c r="V55" s="7" t="inlineStr"/>
+      <c r="W55" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3796,7 +4165,12 @@
       <c r="O56" s="7" t="inlineStr"/>
       <c r="P56" s="7" t="inlineStr"/>
       <c r="Q56" s="7" t="inlineStr"/>
-      <c r="R56" s="7" t="inlineStr">
+      <c r="R56" s="7" t="inlineStr"/>
+      <c r="S56" s="7" t="inlineStr"/>
+      <c r="T56" s="7" t="inlineStr"/>
+      <c r="U56" s="7" t="inlineStr"/>
+      <c r="V56" s="7" t="inlineStr"/>
+      <c r="W56" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3850,7 +4224,12 @@
       <c r="O57" s="7" t="inlineStr"/>
       <c r="P57" s="7" t="inlineStr"/>
       <c r="Q57" s="7" t="inlineStr"/>
-      <c r="R57" s="7" t="inlineStr">
+      <c r="R57" s="7" t="inlineStr"/>
+      <c r="S57" s="7" t="inlineStr"/>
+      <c r="T57" s="7" t="inlineStr"/>
+      <c r="U57" s="7" t="inlineStr"/>
+      <c r="V57" s="7" t="inlineStr"/>
+      <c r="W57" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3898,7 +4277,12 @@
       <c r="O58" s="7" t="inlineStr"/>
       <c r="P58" s="7" t="inlineStr"/>
       <c r="Q58" s="7" t="inlineStr"/>
-      <c r="R58" s="7" t="inlineStr">
+      <c r="R58" s="7" t="inlineStr"/>
+      <c r="S58" s="7" t="inlineStr"/>
+      <c r="T58" s="7" t="inlineStr"/>
+      <c r="U58" s="7" t="inlineStr"/>
+      <c r="V58" s="7" t="inlineStr"/>
+      <c r="W58" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -3954,7 +4338,12 @@
       <c r="O59" s="7" t="inlineStr"/>
       <c r="P59" s="7" t="inlineStr"/>
       <c r="Q59" s="7" t="inlineStr"/>
-      <c r="R59" s="7" t="inlineStr">
+      <c r="R59" s="7" t="inlineStr"/>
+      <c r="S59" s="7" t="inlineStr"/>
+      <c r="T59" s="7" t="inlineStr"/>
+      <c r="U59" s="7" t="inlineStr"/>
+      <c r="V59" s="7" t="inlineStr"/>
+      <c r="W59" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4003,7 +4392,12 @@
       <c r="O60" s="7" t="inlineStr"/>
       <c r="P60" s="7" t="inlineStr"/>
       <c r="Q60" s="7" t="inlineStr"/>
-      <c r="R60" s="7" t="inlineStr">
+      <c r="R60" s="7" t="inlineStr"/>
+      <c r="S60" s="7" t="inlineStr"/>
+      <c r="T60" s="7" t="inlineStr"/>
+      <c r="U60" s="7" t="inlineStr"/>
+      <c r="V60" s="7" t="inlineStr"/>
+      <c r="W60" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4062,7 +4456,12 @@
       <c r="O61" s="7" t="inlineStr"/>
       <c r="P61" s="7" t="inlineStr"/>
       <c r="Q61" s="7" t="inlineStr"/>
-      <c r="R61" s="7" t="inlineStr">
+      <c r="R61" s="7" t="inlineStr"/>
+      <c r="S61" s="7" t="inlineStr"/>
+      <c r="T61" s="7" t="inlineStr"/>
+      <c r="U61" s="7" t="inlineStr"/>
+      <c r="V61" s="7" t="inlineStr"/>
+      <c r="W61" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4115,7 +4514,12 @@
       <c r="O62" s="7" t="inlineStr"/>
       <c r="P62" s="7" t="inlineStr"/>
       <c r="Q62" s="7" t="inlineStr"/>
-      <c r="R62" s="7" t="inlineStr">
+      <c r="R62" s="7" t="inlineStr"/>
+      <c r="S62" s="7" t="inlineStr"/>
+      <c r="T62" s="7" t="inlineStr"/>
+      <c r="U62" s="7" t="inlineStr"/>
+      <c r="V62" s="7" t="inlineStr"/>
+      <c r="W62" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4176,7 +4580,12 @@
       <c r="O63" s="7" t="inlineStr"/>
       <c r="P63" s="7" t="inlineStr"/>
       <c r="Q63" s="7" t="inlineStr"/>
-      <c r="R63" s="7" t="inlineStr">
+      <c r="R63" s="7" t="inlineStr"/>
+      <c r="S63" s="7" t="inlineStr"/>
+      <c r="T63" s="7" t="inlineStr"/>
+      <c r="U63" s="7" t="inlineStr"/>
+      <c r="V63" s="7" t="inlineStr"/>
+      <c r="W63" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4233,7 +4642,12 @@
       <c r="O64" s="7" t="inlineStr"/>
       <c r="P64" s="7" t="inlineStr"/>
       <c r="Q64" s="7" t="inlineStr"/>
-      <c r="R64" s="7" t="inlineStr">
+      <c r="R64" s="7" t="inlineStr"/>
+      <c r="S64" s="7" t="inlineStr"/>
+      <c r="T64" s="7" t="inlineStr"/>
+      <c r="U64" s="7" t="inlineStr"/>
+      <c r="V64" s="7" t="inlineStr"/>
+      <c r="W64" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4281,7 +4695,12 @@
       <c r="O65" s="7" t="inlineStr"/>
       <c r="P65" s="7" t="inlineStr"/>
       <c r="Q65" s="7" t="inlineStr"/>
-      <c r="R65" s="7" t="inlineStr">
+      <c r="R65" s="7" t="inlineStr"/>
+      <c r="S65" s="7" t="inlineStr"/>
+      <c r="T65" s="7" t="inlineStr"/>
+      <c r="U65" s="7" t="inlineStr"/>
+      <c r="V65" s="7" t="inlineStr"/>
+      <c r="W65" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4333,7 +4752,12 @@
       <c r="O66" s="7" t="inlineStr"/>
       <c r="P66" s="7" t="inlineStr"/>
       <c r="Q66" s="7" t="inlineStr"/>
-      <c r="R66" s="7" t="inlineStr">
+      <c r="R66" s="7" t="inlineStr"/>
+      <c r="S66" s="7" t="inlineStr"/>
+      <c r="T66" s="7" t="inlineStr"/>
+      <c r="U66" s="7" t="inlineStr"/>
+      <c r="V66" s="7" t="inlineStr"/>
+      <c r="W66" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4389,7 +4813,12 @@
       <c r="O67" s="7" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr"/>
       <c r="Q67" s="7" t="inlineStr"/>
-      <c r="R67" s="7" t="inlineStr">
+      <c r="R67" s="7" t="inlineStr"/>
+      <c r="S67" s="7" t="inlineStr"/>
+      <c r="T67" s="7" t="inlineStr"/>
+      <c r="U67" s="7" t="inlineStr"/>
+      <c r="V67" s="7" t="inlineStr"/>
+      <c r="W67" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4443,7 +4872,12 @@
       <c r="O68" s="7" t="inlineStr"/>
       <c r="P68" s="7" t="inlineStr"/>
       <c r="Q68" s="7" t="inlineStr"/>
-      <c r="R68" s="7" t="inlineStr">
+      <c r="R68" s="7" t="inlineStr"/>
+      <c r="S68" s="7" t="inlineStr"/>
+      <c r="T68" s="7" t="inlineStr"/>
+      <c r="U68" s="7" t="inlineStr"/>
+      <c r="V68" s="7" t="inlineStr"/>
+      <c r="W68" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4496,7 +4930,12 @@
       <c r="O69" s="7" t="inlineStr"/>
       <c r="P69" s="7" t="inlineStr"/>
       <c r="Q69" s="7" t="inlineStr"/>
-      <c r="R69" s="7" t="inlineStr">
+      <c r="R69" s="7" t="inlineStr"/>
+      <c r="S69" s="7" t="inlineStr"/>
+      <c r="T69" s="7" t="inlineStr"/>
+      <c r="U69" s="7" t="inlineStr"/>
+      <c r="V69" s="7" t="inlineStr"/>
+      <c r="W69" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4547,7 +4986,12 @@
       <c r="O70" s="7" t="inlineStr"/>
       <c r="P70" s="7" t="inlineStr"/>
       <c r="Q70" s="7" t="inlineStr"/>
-      <c r="R70" s="7" t="inlineStr">
+      <c r="R70" s="7" t="inlineStr"/>
+      <c r="S70" s="7" t="inlineStr"/>
+      <c r="T70" s="7" t="inlineStr"/>
+      <c r="U70" s="7" t="inlineStr"/>
+      <c r="V70" s="7" t="inlineStr"/>
+      <c r="W70" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4599,7 +5043,12 @@
       <c r="O71" s="7" t="inlineStr"/>
       <c r="P71" s="7" t="inlineStr"/>
       <c r="Q71" s="7" t="inlineStr"/>
-      <c r="R71" s="7" t="inlineStr">
+      <c r="R71" s="7" t="inlineStr"/>
+      <c r="S71" s="7" t="inlineStr"/>
+      <c r="T71" s="7" t="inlineStr"/>
+      <c r="U71" s="7" t="inlineStr"/>
+      <c r="V71" s="7" t="inlineStr"/>
+      <c r="W71" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4658,7 +5107,12 @@
       <c r="O72" s="7" t="inlineStr"/>
       <c r="P72" s="7" t="inlineStr"/>
       <c r="Q72" s="7" t="inlineStr"/>
-      <c r="R72" s="7" t="inlineStr">
+      <c r="R72" s="7" t="inlineStr"/>
+      <c r="S72" s="7" t="inlineStr"/>
+      <c r="T72" s="7" t="inlineStr"/>
+      <c r="U72" s="7" t="inlineStr"/>
+      <c r="V72" s="7" t="inlineStr"/>
+      <c r="W72" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4710,7 +5164,12 @@
       <c r="O73" s="7" t="inlineStr"/>
       <c r="P73" s="7" t="inlineStr"/>
       <c r="Q73" s="7" t="inlineStr"/>
-      <c r="R73" s="7" t="inlineStr">
+      <c r="R73" s="7" t="inlineStr"/>
+      <c r="S73" s="7" t="inlineStr"/>
+      <c r="T73" s="7" t="inlineStr"/>
+      <c r="U73" s="7" t="inlineStr"/>
+      <c r="V73" s="7" t="inlineStr"/>
+      <c r="W73" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4758,7 +5217,12 @@
       <c r="O74" s="7" t="inlineStr"/>
       <c r="P74" s="7" t="inlineStr"/>
       <c r="Q74" s="7" t="inlineStr"/>
-      <c r="R74" s="7" t="inlineStr">
+      <c r="R74" s="7" t="inlineStr"/>
+      <c r="S74" s="7" t="inlineStr"/>
+      <c r="T74" s="7" t="inlineStr"/>
+      <c r="U74" s="7" t="inlineStr"/>
+      <c r="V74" s="7" t="inlineStr"/>
+      <c r="W74" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4816,7 +5280,12 @@
       <c r="O75" s="7" t="inlineStr"/>
       <c r="P75" s="7" t="inlineStr"/>
       <c r="Q75" s="7" t="inlineStr"/>
-      <c r="R75" s="7" t="inlineStr">
+      <c r="R75" s="7" t="inlineStr"/>
+      <c r="S75" s="7" t="inlineStr"/>
+      <c r="T75" s="7" t="inlineStr"/>
+      <c r="U75" s="7" t="inlineStr"/>
+      <c r="V75" s="7" t="inlineStr"/>
+      <c r="W75" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4871,7 +5340,12 @@
       <c r="O76" s="7" t="inlineStr"/>
       <c r="P76" s="7" t="inlineStr"/>
       <c r="Q76" s="7" t="inlineStr"/>
-      <c r="R76" s="7" t="inlineStr">
+      <c r="R76" s="7" t="inlineStr"/>
+      <c r="S76" s="7" t="inlineStr"/>
+      <c r="T76" s="7" t="inlineStr"/>
+      <c r="U76" s="7" t="inlineStr"/>
+      <c r="V76" s="7" t="inlineStr"/>
+      <c r="W76" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4919,7 +5393,12 @@
       <c r="O77" s="7" t="inlineStr"/>
       <c r="P77" s="7" t="inlineStr"/>
       <c r="Q77" s="7" t="inlineStr"/>
-      <c r="R77" s="7" t="inlineStr">
+      <c r="R77" s="7" t="inlineStr"/>
+      <c r="S77" s="7" t="inlineStr"/>
+      <c r="T77" s="7" t="inlineStr"/>
+      <c r="U77" s="7" t="inlineStr"/>
+      <c r="V77" s="7" t="inlineStr"/>
+      <c r="W77" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -4971,7 +5450,12 @@
       <c r="O78" s="7" t="inlineStr"/>
       <c r="P78" s="7" t="inlineStr"/>
       <c r="Q78" s="7" t="inlineStr"/>
-      <c r="R78" s="7" t="inlineStr">
+      <c r="R78" s="7" t="inlineStr"/>
+      <c r="S78" s="7" t="inlineStr"/>
+      <c r="T78" s="7" t="inlineStr"/>
+      <c r="U78" s="7" t="inlineStr"/>
+      <c r="V78" s="7" t="inlineStr"/>
+      <c r="W78" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5019,7 +5503,12 @@
       <c r="O79" s="7" t="inlineStr"/>
       <c r="P79" s="7" t="inlineStr"/>
       <c r="Q79" s="7" t="inlineStr"/>
-      <c r="R79" s="7" t="inlineStr">
+      <c r="R79" s="7" t="inlineStr"/>
+      <c r="S79" s="7" t="inlineStr"/>
+      <c r="T79" s="7" t="inlineStr"/>
+      <c r="U79" s="7" t="inlineStr"/>
+      <c r="V79" s="7" t="inlineStr"/>
+      <c r="W79" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5071,7 +5560,12 @@
       <c r="O80" s="7" t="inlineStr"/>
       <c r="P80" s="7" t="inlineStr"/>
       <c r="Q80" s="7" t="inlineStr"/>
-      <c r="R80" s="7" t="inlineStr">
+      <c r="R80" s="7" t="inlineStr"/>
+      <c r="S80" s="7" t="inlineStr"/>
+      <c r="T80" s="7" t="inlineStr"/>
+      <c r="U80" s="7" t="inlineStr"/>
+      <c r="V80" s="7" t="inlineStr"/>
+      <c r="W80" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5119,7 +5613,12 @@
       <c r="O81" s="7" t="inlineStr"/>
       <c r="P81" s="7" t="inlineStr"/>
       <c r="Q81" s="7" t="inlineStr"/>
-      <c r="R81" s="7" t="inlineStr">
+      <c r="R81" s="7" t="inlineStr"/>
+      <c r="S81" s="7" t="inlineStr"/>
+      <c r="T81" s="7" t="inlineStr"/>
+      <c r="U81" s="7" t="inlineStr"/>
+      <c r="V81" s="7" t="inlineStr"/>
+      <c r="W81" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5171,7 +5670,12 @@
       <c r="O82" s="7" t="inlineStr"/>
       <c r="P82" s="7" t="inlineStr"/>
       <c r="Q82" s="7" t="inlineStr"/>
-      <c r="R82" s="7" t="inlineStr">
+      <c r="R82" s="7" t="inlineStr"/>
+      <c r="S82" s="7" t="inlineStr"/>
+      <c r="T82" s="7" t="inlineStr"/>
+      <c r="U82" s="7" t="inlineStr"/>
+      <c r="V82" s="7" t="inlineStr"/>
+      <c r="W82" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5239,7 +5743,12 @@
       <c r="O83" s="7" t="inlineStr"/>
       <c r="P83" s="7" t="inlineStr"/>
       <c r="Q83" s="7" t="inlineStr"/>
-      <c r="R83" s="7" t="inlineStr">
+      <c r="R83" s="7" t="inlineStr"/>
+      <c r="S83" s="7" t="inlineStr"/>
+      <c r="T83" s="7" t="inlineStr"/>
+      <c r="U83" s="7" t="inlineStr"/>
+      <c r="V83" s="7" t="inlineStr"/>
+      <c r="W83" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5288,7 +5797,12 @@
       <c r="O84" s="7" t="inlineStr"/>
       <c r="P84" s="7" t="inlineStr"/>
       <c r="Q84" s="7" t="inlineStr"/>
-      <c r="R84" s="7" t="inlineStr">
+      <c r="R84" s="7" t="inlineStr"/>
+      <c r="S84" s="7" t="inlineStr"/>
+      <c r="T84" s="7" t="inlineStr"/>
+      <c r="U84" s="7" t="inlineStr"/>
+      <c r="V84" s="7" t="inlineStr"/>
+      <c r="W84" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5341,7 +5855,12 @@
       <c r="O85" s="7" t="inlineStr"/>
       <c r="P85" s="7" t="inlineStr"/>
       <c r="Q85" s="7" t="inlineStr"/>
-      <c r="R85" s="7" t="inlineStr">
+      <c r="R85" s="7" t="inlineStr"/>
+      <c r="S85" s="7" t="inlineStr"/>
+      <c r="T85" s="7" t="inlineStr"/>
+      <c r="U85" s="7" t="inlineStr"/>
+      <c r="V85" s="7" t="inlineStr"/>
+      <c r="W85" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5393,7 +5912,12 @@
       <c r="O86" s="7" t="inlineStr"/>
       <c r="P86" s="7" t="inlineStr"/>
       <c r="Q86" s="7" t="inlineStr"/>
-      <c r="R86" s="7" t="inlineStr">
+      <c r="R86" s="7" t="inlineStr"/>
+      <c r="S86" s="7" t="inlineStr"/>
+      <c r="T86" s="7" t="inlineStr"/>
+      <c r="U86" s="7" t="inlineStr"/>
+      <c r="V86" s="7" t="inlineStr"/>
+      <c r="W86" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5443,7 +5967,12 @@
       <c r="O87" s="7" t="inlineStr"/>
       <c r="P87" s="7" t="inlineStr"/>
       <c r="Q87" s="7" t="inlineStr"/>
-      <c r="R87" s="7" t="inlineStr">
+      <c r="R87" s="7" t="inlineStr"/>
+      <c r="S87" s="7" t="inlineStr"/>
+      <c r="T87" s="7" t="inlineStr"/>
+      <c r="U87" s="7" t="inlineStr"/>
+      <c r="V87" s="7" t="inlineStr"/>
+      <c r="W87" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5496,7 +6025,12 @@
       <c r="O88" s="7" t="inlineStr"/>
       <c r="P88" s="7" t="inlineStr"/>
       <c r="Q88" s="7" t="inlineStr"/>
-      <c r="R88" s="7" t="inlineStr">
+      <c r="R88" s="7" t="inlineStr"/>
+      <c r="S88" s="7" t="inlineStr"/>
+      <c r="T88" s="7" t="inlineStr"/>
+      <c r="U88" s="7" t="inlineStr"/>
+      <c r="V88" s="7" t="inlineStr"/>
+      <c r="W88" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5553,7 +6087,12 @@
       <c r="O89" s="7" t="inlineStr"/>
       <c r="P89" s="7" t="inlineStr"/>
       <c r="Q89" s="7" t="inlineStr"/>
-      <c r="R89" s="7" t="inlineStr">
+      <c r="R89" s="7" t="inlineStr"/>
+      <c r="S89" s="7" t="inlineStr"/>
+      <c r="T89" s="7" t="inlineStr"/>
+      <c r="U89" s="7" t="inlineStr"/>
+      <c r="V89" s="7" t="inlineStr"/>
+      <c r="W89" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5608,7 +6147,12 @@
       <c r="O90" s="7" t="inlineStr"/>
       <c r="P90" s="7" t="inlineStr"/>
       <c r="Q90" s="7" t="inlineStr"/>
-      <c r="R90" s="7" t="inlineStr">
+      <c r="R90" s="7" t="inlineStr"/>
+      <c r="S90" s="7" t="inlineStr"/>
+      <c r="T90" s="7" t="inlineStr"/>
+      <c r="U90" s="7" t="inlineStr"/>
+      <c r="V90" s="7" t="inlineStr"/>
+      <c r="W90" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5665,7 +6209,12 @@
       <c r="O91" s="7" t="inlineStr"/>
       <c r="P91" s="7" t="inlineStr"/>
       <c r="Q91" s="7" t="inlineStr"/>
-      <c r="R91" s="7" t="inlineStr">
+      <c r="R91" s="7" t="inlineStr"/>
+      <c r="S91" s="7" t="inlineStr"/>
+      <c r="T91" s="7" t="inlineStr"/>
+      <c r="U91" s="7" t="inlineStr"/>
+      <c r="V91" s="7" t="inlineStr"/>
+      <c r="W91" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5718,7 +6267,12 @@
       <c r="O92" s="7" t="inlineStr"/>
       <c r="P92" s="7" t="inlineStr"/>
       <c r="Q92" s="7" t="inlineStr"/>
-      <c r="R92" s="7" t="inlineStr">
+      <c r="R92" s="7" t="inlineStr"/>
+      <c r="S92" s="7" t="inlineStr"/>
+      <c r="T92" s="7" t="inlineStr"/>
+      <c r="U92" s="7" t="inlineStr"/>
+      <c r="V92" s="7" t="inlineStr"/>
+      <c r="W92" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5766,7 +6320,12 @@
       <c r="O93" s="7" t="inlineStr"/>
       <c r="P93" s="7" t="inlineStr"/>
       <c r="Q93" s="7" t="inlineStr"/>
-      <c r="R93" s="7" t="inlineStr">
+      <c r="R93" s="7" t="inlineStr"/>
+      <c r="S93" s="7" t="inlineStr"/>
+      <c r="T93" s="7" t="inlineStr"/>
+      <c r="U93" s="7" t="inlineStr"/>
+      <c r="V93" s="7" t="inlineStr"/>
+      <c r="W93" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5818,7 +6377,12 @@
       <c r="O94" s="7" t="inlineStr"/>
       <c r="P94" s="7" t="inlineStr"/>
       <c r="Q94" s="7" t="inlineStr"/>
-      <c r="R94" s="7" t="inlineStr">
+      <c r="R94" s="7" t="inlineStr"/>
+      <c r="S94" s="7" t="inlineStr"/>
+      <c r="T94" s="7" t="inlineStr"/>
+      <c r="U94" s="7" t="inlineStr"/>
+      <c r="V94" s="7" t="inlineStr"/>
+      <c r="W94" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5875,7 +6439,12 @@
       <c r="O95" s="7" t="inlineStr"/>
       <c r="P95" s="7" t="inlineStr"/>
       <c r="Q95" s="7" t="inlineStr"/>
-      <c r="R95" s="7" t="inlineStr">
+      <c r="R95" s="7" t="inlineStr"/>
+      <c r="S95" s="7" t="inlineStr"/>
+      <c r="T95" s="7" t="inlineStr"/>
+      <c r="U95" s="7" t="inlineStr"/>
+      <c r="V95" s="7" t="inlineStr"/>
+      <c r="W95" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5929,7 +6498,12 @@
       <c r="O96" s="7" t="inlineStr"/>
       <c r="P96" s="7" t="inlineStr"/>
       <c r="Q96" s="7" t="inlineStr"/>
-      <c r="R96" s="7" t="inlineStr">
+      <c r="R96" s="7" t="inlineStr"/>
+      <c r="S96" s="7" t="inlineStr"/>
+      <c r="T96" s="7" t="inlineStr"/>
+      <c r="U96" s="7" t="inlineStr"/>
+      <c r="V96" s="7" t="inlineStr"/>
+      <c r="W96" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -5979,7 +6553,12 @@
       <c r="O97" s="7" t="inlineStr"/>
       <c r="P97" s="7" t="inlineStr"/>
       <c r="Q97" s="7" t="inlineStr"/>
-      <c r="R97" s="7" t="inlineStr">
+      <c r="R97" s="7" t="inlineStr"/>
+      <c r="S97" s="7" t="inlineStr"/>
+      <c r="T97" s="7" t="inlineStr"/>
+      <c r="U97" s="7" t="inlineStr"/>
+      <c r="V97" s="7" t="inlineStr"/>
+      <c r="W97" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6034,7 +6613,12 @@
       <c r="O98" s="7" t="inlineStr"/>
       <c r="P98" s="7" t="inlineStr"/>
       <c r="Q98" s="7" t="inlineStr"/>
-      <c r="R98" s="7" t="inlineStr">
+      <c r="R98" s="7" t="inlineStr"/>
+      <c r="S98" s="7" t="inlineStr"/>
+      <c r="T98" s="7" t="inlineStr"/>
+      <c r="U98" s="7" t="inlineStr"/>
+      <c r="V98" s="7" t="inlineStr"/>
+      <c r="W98" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6082,7 +6666,12 @@
       <c r="O99" s="7" t="inlineStr"/>
       <c r="P99" s="7" t="inlineStr"/>
       <c r="Q99" s="7" t="inlineStr"/>
-      <c r="R99" s="7" t="inlineStr">
+      <c r="R99" s="7" t="inlineStr"/>
+      <c r="S99" s="7" t="inlineStr"/>
+      <c r="T99" s="7" t="inlineStr"/>
+      <c r="U99" s="7" t="inlineStr"/>
+      <c r="V99" s="7" t="inlineStr"/>
+      <c r="W99" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6130,7 +6719,12 @@
       <c r="O100" s="7" t="inlineStr"/>
       <c r="P100" s="7" t="inlineStr"/>
       <c r="Q100" s="7" t="inlineStr"/>
-      <c r="R100" s="7" t="inlineStr">
+      <c r="R100" s="7" t="inlineStr"/>
+      <c r="S100" s="7" t="inlineStr"/>
+      <c r="T100" s="7" t="inlineStr"/>
+      <c r="U100" s="7" t="inlineStr"/>
+      <c r="V100" s="7" t="inlineStr"/>
+      <c r="W100" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6186,7 +6780,12 @@
       <c r="O101" s="7" t="inlineStr"/>
       <c r="P101" s="7" t="inlineStr"/>
       <c r="Q101" s="7" t="inlineStr"/>
-      <c r="R101" s="7" t="inlineStr">
+      <c r="R101" s="7" t="inlineStr"/>
+      <c r="S101" s="7" t="inlineStr"/>
+      <c r="T101" s="7" t="inlineStr"/>
+      <c r="U101" s="7" t="inlineStr"/>
+      <c r="V101" s="7" t="inlineStr"/>
+      <c r="W101" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6241,7 +6840,12 @@
       <c r="O102" s="7" t="inlineStr"/>
       <c r="P102" s="7" t="inlineStr"/>
       <c r="Q102" s="7" t="inlineStr"/>
-      <c r="R102" s="7" t="inlineStr">
+      <c r="R102" s="7" t="inlineStr"/>
+      <c r="S102" s="7" t="inlineStr"/>
+      <c r="T102" s="7" t="inlineStr"/>
+      <c r="U102" s="7" t="inlineStr"/>
+      <c r="V102" s="7" t="inlineStr"/>
+      <c r="W102" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6294,7 +6898,12 @@
       <c r="O103" s="7" t="inlineStr"/>
       <c r="P103" s="7" t="inlineStr"/>
       <c r="Q103" s="7" t="inlineStr"/>
-      <c r="R103" s="7" t="inlineStr">
+      <c r="R103" s="7" t="inlineStr"/>
+      <c r="S103" s="7" t="inlineStr"/>
+      <c r="T103" s="7" t="inlineStr"/>
+      <c r="U103" s="7" t="inlineStr"/>
+      <c r="V103" s="7" t="inlineStr"/>
+      <c r="W103" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6345,7 +6954,12 @@
       <c r="O104" s="7" t="inlineStr"/>
       <c r="P104" s="7" t="inlineStr"/>
       <c r="Q104" s="7" t="inlineStr"/>
-      <c r="R104" s="7" t="inlineStr">
+      <c r="R104" s="7" t="inlineStr"/>
+      <c r="S104" s="7" t="inlineStr"/>
+      <c r="T104" s="7" t="inlineStr"/>
+      <c r="U104" s="7" t="inlineStr"/>
+      <c r="V104" s="7" t="inlineStr"/>
+      <c r="W104" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6400,7 +7014,12 @@
       <c r="O105" s="7" t="inlineStr"/>
       <c r="P105" s="7" t="inlineStr"/>
       <c r="Q105" s="7" t="inlineStr"/>
-      <c r="R105" s="7" t="inlineStr">
+      <c r="R105" s="7" t="inlineStr"/>
+      <c r="S105" s="7" t="inlineStr"/>
+      <c r="T105" s="7" t="inlineStr"/>
+      <c r="U105" s="7" t="inlineStr"/>
+      <c r="V105" s="7" t="inlineStr"/>
+      <c r="W105" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6452,7 +7071,12 @@
       <c r="O106" s="7" t="inlineStr"/>
       <c r="P106" s="7" t="inlineStr"/>
       <c r="Q106" s="7" t="inlineStr"/>
-      <c r="R106" s="7" t="inlineStr">
+      <c r="R106" s="7" t="inlineStr"/>
+      <c r="S106" s="7" t="inlineStr"/>
+      <c r="T106" s="7" t="inlineStr"/>
+      <c r="U106" s="7" t="inlineStr"/>
+      <c r="V106" s="7" t="inlineStr"/>
+      <c r="W106" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6507,7 +7131,12 @@
       <c r="O107" s="7" t="inlineStr"/>
       <c r="P107" s="7" t="inlineStr"/>
       <c r="Q107" s="7" t="inlineStr"/>
-      <c r="R107" s="7" t="inlineStr">
+      <c r="R107" s="7" t="inlineStr"/>
+      <c r="S107" s="7" t="inlineStr"/>
+      <c r="T107" s="7" t="inlineStr"/>
+      <c r="U107" s="7" t="inlineStr"/>
+      <c r="V107" s="7" t="inlineStr"/>
+      <c r="W107" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6555,7 +7184,12 @@
       <c r="O108" s="7" t="inlineStr"/>
       <c r="P108" s="7" t="inlineStr"/>
       <c r="Q108" s="7" t="inlineStr"/>
-      <c r="R108" s="7" t="inlineStr">
+      <c r="R108" s="7" t="inlineStr"/>
+      <c r="S108" s="7" t="inlineStr"/>
+      <c r="T108" s="7" t="inlineStr"/>
+      <c r="U108" s="7" t="inlineStr"/>
+      <c r="V108" s="7" t="inlineStr"/>
+      <c r="W108" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6607,7 +7241,12 @@
       <c r="O109" s="7" t="inlineStr"/>
       <c r="P109" s="7" t="inlineStr"/>
       <c r="Q109" s="7" t="inlineStr"/>
-      <c r="R109" s="7" t="inlineStr">
+      <c r="R109" s="7" t="inlineStr"/>
+      <c r="S109" s="7" t="inlineStr"/>
+      <c r="T109" s="7" t="inlineStr"/>
+      <c r="U109" s="7" t="inlineStr"/>
+      <c r="V109" s="7" t="inlineStr"/>
+      <c r="W109" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6655,7 +7294,12 @@
       <c r="O110" s="7" t="inlineStr"/>
       <c r="P110" s="7" t="inlineStr"/>
       <c r="Q110" s="7" t="inlineStr"/>
-      <c r="R110" s="7" t="inlineStr">
+      <c r="R110" s="7" t="inlineStr"/>
+      <c r="S110" s="7" t="inlineStr"/>
+      <c r="T110" s="7" t="inlineStr"/>
+      <c r="U110" s="7" t="inlineStr"/>
+      <c r="V110" s="7" t="inlineStr"/>
+      <c r="W110" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6711,7 +7355,12 @@
       <c r="O111" s="7" t="inlineStr"/>
       <c r="P111" s="7" t="inlineStr"/>
       <c r="Q111" s="7" t="inlineStr"/>
-      <c r="R111" s="7" t="inlineStr">
+      <c r="R111" s="7" t="inlineStr"/>
+      <c r="S111" s="7" t="inlineStr"/>
+      <c r="T111" s="7" t="inlineStr"/>
+      <c r="U111" s="7" t="inlineStr"/>
+      <c r="V111" s="7" t="inlineStr"/>
+      <c r="W111" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6761,7 +7410,12 @@
       <c r="O112" s="7" t="inlineStr"/>
       <c r="P112" s="7" t="inlineStr"/>
       <c r="Q112" s="7" t="inlineStr"/>
-      <c r="R112" s="7" t="inlineStr">
+      <c r="R112" s="7" t="inlineStr"/>
+      <c r="S112" s="7" t="inlineStr"/>
+      <c r="T112" s="7" t="inlineStr"/>
+      <c r="U112" s="7" t="inlineStr"/>
+      <c r="V112" s="7" t="inlineStr"/>
+      <c r="W112" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6809,7 +7463,12 @@
       <c r="O113" s="7" t="inlineStr"/>
       <c r="P113" s="7" t="inlineStr"/>
       <c r="Q113" s="7" t="inlineStr"/>
-      <c r="R113" s="7" t="inlineStr">
+      <c r="R113" s="7" t="inlineStr"/>
+      <c r="S113" s="7" t="inlineStr"/>
+      <c r="T113" s="7" t="inlineStr"/>
+      <c r="U113" s="7" t="inlineStr"/>
+      <c r="V113" s="7" t="inlineStr"/>
+      <c r="W113" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6864,7 +7523,12 @@
       <c r="O114" s="7" t="inlineStr"/>
       <c r="P114" s="7" t="inlineStr"/>
       <c r="Q114" s="7" t="inlineStr"/>
-      <c r="R114" s="7" t="inlineStr">
+      <c r="R114" s="7" t="inlineStr"/>
+      <c r="S114" s="7" t="inlineStr"/>
+      <c r="T114" s="7" t="inlineStr"/>
+      <c r="U114" s="7" t="inlineStr"/>
+      <c r="V114" s="7" t="inlineStr"/>
+      <c r="W114" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6922,7 +7586,12 @@
       <c r="O115" s="7" t="inlineStr"/>
       <c r="P115" s="7" t="inlineStr"/>
       <c r="Q115" s="7" t="inlineStr"/>
-      <c r="R115" s="7" t="inlineStr">
+      <c r="R115" s="7" t="inlineStr"/>
+      <c r="S115" s="7" t="inlineStr"/>
+      <c r="T115" s="7" t="inlineStr"/>
+      <c r="U115" s="7" t="inlineStr"/>
+      <c r="V115" s="7" t="inlineStr"/>
+      <c r="W115" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -6970,7 +7639,12 @@
       <c r="O116" s="7" t="inlineStr"/>
       <c r="P116" s="7" t="inlineStr"/>
       <c r="Q116" s="7" t="inlineStr"/>
-      <c r="R116" s="7" t="inlineStr">
+      <c r="R116" s="7" t="inlineStr"/>
+      <c r="S116" s="7" t="inlineStr"/>
+      <c r="T116" s="7" t="inlineStr"/>
+      <c r="U116" s="7" t="inlineStr"/>
+      <c r="V116" s="7" t="inlineStr"/>
+      <c r="W116" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7027,7 +7701,12 @@
       <c r="O117" s="7" t="inlineStr"/>
       <c r="P117" s="7" t="inlineStr"/>
       <c r="Q117" s="7" t="inlineStr"/>
-      <c r="R117" s="7" t="inlineStr">
+      <c r="R117" s="7" t="inlineStr"/>
+      <c r="S117" s="7" t="inlineStr"/>
+      <c r="T117" s="7" t="inlineStr"/>
+      <c r="U117" s="7" t="inlineStr"/>
+      <c r="V117" s="7" t="inlineStr"/>
+      <c r="W117" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7075,7 +7754,12 @@
       <c r="O118" s="7" t="inlineStr"/>
       <c r="P118" s="7" t="inlineStr"/>
       <c r="Q118" s="7" t="inlineStr"/>
-      <c r="R118" s="7" t="inlineStr">
+      <c r="R118" s="7" t="inlineStr"/>
+      <c r="S118" s="7" t="inlineStr"/>
+      <c r="T118" s="7" t="inlineStr"/>
+      <c r="U118" s="7" t="inlineStr"/>
+      <c r="V118" s="7" t="inlineStr"/>
+      <c r="W118" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7138,7 +7822,12 @@
       <c r="O119" s="7" t="inlineStr"/>
       <c r="P119" s="7" t="inlineStr"/>
       <c r="Q119" s="7" t="inlineStr"/>
-      <c r="R119" s="7" t="inlineStr">
+      <c r="R119" s="7" t="inlineStr"/>
+      <c r="S119" s="7" t="inlineStr"/>
+      <c r="T119" s="7" t="inlineStr"/>
+      <c r="U119" s="7" t="inlineStr"/>
+      <c r="V119" s="7" t="inlineStr"/>
+      <c r="W119" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7194,7 +7883,12 @@
       <c r="O120" s="7" t="inlineStr"/>
       <c r="P120" s="7" t="inlineStr"/>
       <c r="Q120" s="7" t="inlineStr"/>
-      <c r="R120" s="7" t="inlineStr">
+      <c r="R120" s="7" t="inlineStr"/>
+      <c r="S120" s="7" t="inlineStr"/>
+      <c r="T120" s="7" t="inlineStr"/>
+      <c r="U120" s="7" t="inlineStr"/>
+      <c r="V120" s="7" t="inlineStr"/>
+      <c r="W120" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7243,7 +7937,12 @@
       <c r="O121" s="7" t="inlineStr"/>
       <c r="P121" s="7" t="inlineStr"/>
       <c r="Q121" s="7" t="inlineStr"/>
-      <c r="R121" s="7" t="inlineStr">
+      <c r="R121" s="7" t="inlineStr"/>
+      <c r="S121" s="7" t="inlineStr"/>
+      <c r="T121" s="7" t="inlineStr"/>
+      <c r="U121" s="7" t="inlineStr"/>
+      <c r="V121" s="7" t="inlineStr"/>
+      <c r="W121" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7291,7 +7990,12 @@
       <c r="O122" s="7" t="inlineStr"/>
       <c r="P122" s="7" t="inlineStr"/>
       <c r="Q122" s="7" t="inlineStr"/>
-      <c r="R122" s="7" t="inlineStr">
+      <c r="R122" s="7" t="inlineStr"/>
+      <c r="S122" s="7" t="inlineStr"/>
+      <c r="T122" s="7" t="inlineStr"/>
+      <c r="U122" s="7" t="inlineStr"/>
+      <c r="V122" s="7" t="inlineStr"/>
+      <c r="W122" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7357,7 +8061,12 @@
       <c r="O123" s="7" t="inlineStr"/>
       <c r="P123" s="7" t="inlineStr"/>
       <c r="Q123" s="7" t="inlineStr"/>
-      <c r="R123" s="7" t="inlineStr">
+      <c r="R123" s="7" t="inlineStr"/>
+      <c r="S123" s="7" t="inlineStr"/>
+      <c r="T123" s="7" t="inlineStr"/>
+      <c r="U123" s="7" t="inlineStr"/>
+      <c r="V123" s="7" t="inlineStr"/>
+      <c r="W123" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7410,7 +8119,12 @@
       <c r="O124" s="7" t="inlineStr"/>
       <c r="P124" s="7" t="inlineStr"/>
       <c r="Q124" s="7" t="inlineStr"/>
-      <c r="R124" s="7" t="inlineStr">
+      <c r="R124" s="7" t="inlineStr"/>
+      <c r="S124" s="7" t="inlineStr"/>
+      <c r="T124" s="7" t="inlineStr"/>
+      <c r="U124" s="7" t="inlineStr"/>
+      <c r="V124" s="7" t="inlineStr"/>
+      <c r="W124" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7478,7 +8192,12 @@
       <c r="O125" s="7" t="inlineStr"/>
       <c r="P125" s="7" t="inlineStr"/>
       <c r="Q125" s="7" t="inlineStr"/>
-      <c r="R125" s="7" t="inlineStr">
+      <c r="R125" s="7" t="inlineStr"/>
+      <c r="S125" s="7" t="inlineStr"/>
+      <c r="T125" s="7" t="inlineStr"/>
+      <c r="U125" s="7" t="inlineStr"/>
+      <c r="V125" s="7" t="inlineStr"/>
+      <c r="W125" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7533,7 +8252,12 @@
       <c r="O126" s="7" t="inlineStr"/>
       <c r="P126" s="7" t="inlineStr"/>
       <c r="Q126" s="7" t="inlineStr"/>
-      <c r="R126" s="7" t="inlineStr">
+      <c r="R126" s="7" t="inlineStr"/>
+      <c r="S126" s="7" t="inlineStr"/>
+      <c r="T126" s="7" t="inlineStr"/>
+      <c r="U126" s="7" t="inlineStr"/>
+      <c r="V126" s="7" t="inlineStr"/>
+      <c r="W126" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7585,7 +8309,12 @@
       <c r="O127" s="7" t="inlineStr"/>
       <c r="P127" s="7" t="inlineStr"/>
       <c r="Q127" s="7" t="inlineStr"/>
-      <c r="R127" s="7" t="inlineStr">
+      <c r="R127" s="7" t="inlineStr"/>
+      <c r="S127" s="7" t="inlineStr"/>
+      <c r="T127" s="7" t="inlineStr"/>
+      <c r="U127" s="7" t="inlineStr"/>
+      <c r="V127" s="7" t="inlineStr"/>
+      <c r="W127" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7635,7 +8364,12 @@
       <c r="O128" s="7" t="inlineStr"/>
       <c r="P128" s="7" t="inlineStr"/>
       <c r="Q128" s="7" t="inlineStr"/>
-      <c r="R128" s="7" t="inlineStr">
+      <c r="R128" s="7" t="inlineStr"/>
+      <c r="S128" s="7" t="inlineStr"/>
+      <c r="T128" s="7" t="inlineStr"/>
+      <c r="U128" s="7" t="inlineStr"/>
+      <c r="V128" s="7" t="inlineStr"/>
+      <c r="W128" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7686,7 +8420,12 @@
       <c r="O129" s="7" t="inlineStr"/>
       <c r="P129" s="7" t="inlineStr"/>
       <c r="Q129" s="7" t="inlineStr"/>
-      <c r="R129" s="7" t="inlineStr">
+      <c r="R129" s="7" t="inlineStr"/>
+      <c r="S129" s="7" t="inlineStr"/>
+      <c r="T129" s="7" t="inlineStr"/>
+      <c r="U129" s="7" t="inlineStr"/>
+      <c r="V129" s="7" t="inlineStr"/>
+      <c r="W129" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7734,7 +8473,12 @@
       <c r="O130" s="7" t="inlineStr"/>
       <c r="P130" s="7" t="inlineStr"/>
       <c r="Q130" s="7" t="inlineStr"/>
-      <c r="R130" s="7" t="inlineStr">
+      <c r="R130" s="7" t="inlineStr"/>
+      <c r="S130" s="7" t="inlineStr"/>
+      <c r="T130" s="7" t="inlineStr"/>
+      <c r="U130" s="7" t="inlineStr"/>
+      <c r="V130" s="7" t="inlineStr"/>
+      <c r="W130" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7787,7 +8531,12 @@
       <c r="O131" s="7" t="inlineStr"/>
       <c r="P131" s="7" t="inlineStr"/>
       <c r="Q131" s="7" t="inlineStr"/>
-      <c r="R131" s="7" t="inlineStr">
+      <c r="R131" s="7" t="inlineStr"/>
+      <c r="S131" s="7" t="inlineStr"/>
+      <c r="T131" s="7" t="inlineStr"/>
+      <c r="U131" s="7" t="inlineStr"/>
+      <c r="V131" s="7" t="inlineStr"/>
+      <c r="W131" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7845,7 +8594,12 @@
       <c r="O132" s="7" t="inlineStr"/>
       <c r="P132" s="7" t="inlineStr"/>
       <c r="Q132" s="7" t="inlineStr"/>
-      <c r="R132" s="7" t="inlineStr">
+      <c r="R132" s="7" t="inlineStr"/>
+      <c r="S132" s="7" t="inlineStr"/>
+      <c r="T132" s="7" t="inlineStr"/>
+      <c r="U132" s="7" t="inlineStr"/>
+      <c r="V132" s="7" t="inlineStr"/>
+      <c r="W132" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7893,7 +8647,12 @@
       <c r="O133" s="7" t="inlineStr"/>
       <c r="P133" s="7" t="inlineStr"/>
       <c r="Q133" s="7" t="inlineStr"/>
-      <c r="R133" s="7" t="inlineStr">
+      <c r="R133" s="7" t="inlineStr"/>
+      <c r="S133" s="7" t="inlineStr"/>
+      <c r="T133" s="7" t="inlineStr"/>
+      <c r="U133" s="7" t="inlineStr"/>
+      <c r="V133" s="7" t="inlineStr"/>
+      <c r="W133" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7943,7 +8702,12 @@
       <c r="O134" s="7" t="inlineStr"/>
       <c r="P134" s="7" t="inlineStr"/>
       <c r="Q134" s="7" t="inlineStr"/>
-      <c r="R134" s="7" t="inlineStr">
+      <c r="R134" s="7" t="inlineStr"/>
+      <c r="S134" s="7" t="inlineStr"/>
+      <c r="T134" s="7" t="inlineStr"/>
+      <c r="U134" s="7" t="inlineStr"/>
+      <c r="V134" s="7" t="inlineStr"/>
+      <c r="W134" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -7991,7 +8755,12 @@
       <c r="O135" s="7" t="inlineStr"/>
       <c r="P135" s="7" t="inlineStr"/>
       <c r="Q135" s="7" t="inlineStr"/>
-      <c r="R135" s="7" t="inlineStr">
+      <c r="R135" s="7" t="inlineStr"/>
+      <c r="S135" s="7" t="inlineStr"/>
+      <c r="T135" s="7" t="inlineStr"/>
+      <c r="U135" s="7" t="inlineStr"/>
+      <c r="V135" s="7" t="inlineStr"/>
+      <c r="W135" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8049,7 +8818,12 @@
       <c r="O136" s="7" t="inlineStr"/>
       <c r="P136" s="7" t="inlineStr"/>
       <c r="Q136" s="7" t="inlineStr"/>
-      <c r="R136" s="7" t="inlineStr">
+      <c r="R136" s="7" t="inlineStr"/>
+      <c r="S136" s="7" t="inlineStr"/>
+      <c r="T136" s="7" t="inlineStr"/>
+      <c r="U136" s="7" t="inlineStr"/>
+      <c r="V136" s="7" t="inlineStr"/>
+      <c r="W136" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8105,7 +8879,12 @@
       <c r="O137" s="7" t="inlineStr"/>
       <c r="P137" s="7" t="inlineStr"/>
       <c r="Q137" s="7" t="inlineStr"/>
-      <c r="R137" s="7" t="inlineStr">
+      <c r="R137" s="7" t="inlineStr"/>
+      <c r="S137" s="7" t="inlineStr"/>
+      <c r="T137" s="7" t="inlineStr"/>
+      <c r="U137" s="7" t="inlineStr"/>
+      <c r="V137" s="7" t="inlineStr"/>
+      <c r="W137" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8155,7 +8934,12 @@
       <c r="O138" s="7" t="inlineStr"/>
       <c r="P138" s="7" t="inlineStr"/>
       <c r="Q138" s="7" t="inlineStr"/>
-      <c r="R138" s="7" t="inlineStr">
+      <c r="R138" s="7" t="inlineStr"/>
+      <c r="S138" s="7" t="inlineStr"/>
+      <c r="T138" s="7" t="inlineStr"/>
+      <c r="U138" s="7" t="inlineStr"/>
+      <c r="V138" s="7" t="inlineStr"/>
+      <c r="W138" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8204,7 +8988,12 @@
       <c r="O139" s="7" t="inlineStr"/>
       <c r="P139" s="7" t="inlineStr"/>
       <c r="Q139" s="7" t="inlineStr"/>
-      <c r="R139" s="7" t="inlineStr">
+      <c r="R139" s="7" t="inlineStr"/>
+      <c r="S139" s="7" t="inlineStr"/>
+      <c r="T139" s="7" t="inlineStr"/>
+      <c r="U139" s="7" t="inlineStr"/>
+      <c r="V139" s="7" t="inlineStr"/>
+      <c r="W139" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8252,7 +9041,12 @@
       <c r="O140" s="7" t="inlineStr"/>
       <c r="P140" s="7" t="inlineStr"/>
       <c r="Q140" s="7" t="inlineStr"/>
-      <c r="R140" s="7" t="inlineStr">
+      <c r="R140" s="7" t="inlineStr"/>
+      <c r="S140" s="7" t="inlineStr"/>
+      <c r="T140" s="7" t="inlineStr"/>
+      <c r="U140" s="7" t="inlineStr"/>
+      <c r="V140" s="7" t="inlineStr"/>
+      <c r="W140" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8302,7 +9096,12 @@
       <c r="O141" s="7" t="inlineStr"/>
       <c r="P141" s="7" t="inlineStr"/>
       <c r="Q141" s="7" t="inlineStr"/>
-      <c r="R141" s="7" t="inlineStr">
+      <c r="R141" s="7" t="inlineStr"/>
+      <c r="S141" s="7" t="inlineStr"/>
+      <c r="T141" s="7" t="inlineStr"/>
+      <c r="U141" s="7" t="inlineStr"/>
+      <c r="V141" s="7" t="inlineStr"/>
+      <c r="W141" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
@@ -8362,23 +9161,28 @@
       <c r="O142" s="7" t="inlineStr"/>
       <c r="P142" s="7" t="inlineStr"/>
       <c r="Q142" s="7" t="inlineStr"/>
-      <c r="R142" s="7" t="inlineStr">
+      <c r="R142" s="7" t="inlineStr"/>
+      <c r="S142" s="7" t="inlineStr"/>
+      <c r="T142" s="7" t="inlineStr"/>
+      <c r="U142" s="7" t="inlineStr"/>
+      <c r="V142" s="7" t="inlineStr"/>
+      <c r="W142" s="7" t="inlineStr">
         <is>
           <t>unlabeled</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R2"/>
-  <conditionalFormatting sqref="A3:R142">
+  <autoFilter ref="A2:W2"/>
+  <conditionalFormatting sqref="A3:W142">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEFT($R3,7)="labeled"</formula>
+      <formula>LEFT($W3,7)="labeled"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT($R3,16)="needs_discussion"</formula>
+      <formula>LEFT($W3,16)="needs_discussion"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="10">
+  <dataValidations count="15">
     <dataValidation sqref="H3:H142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
       <formula1>='下拉选项'!$A$2:$A$4</formula1>
     </dataValidation>
@@ -8398,16 +9202,31 @@
       <formula1>='下拉选项'!$F$2:$F$4</formula1>
     </dataValidation>
     <dataValidation sqref="N3:N142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
-      <formula1>='下拉选项'!$G$2:$G$5</formula1>
+      <formula1>='下拉选项'!$G$2:$G$4</formula1>
     </dataValidation>
     <dataValidation sqref="O3:O142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
-      <formula1>='下拉选项'!$H$2:$H$5</formula1>
+      <formula1>='下拉选项'!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="P3:P142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
       <formula1>='下拉选项'!$I$2:$I$5</formula1>
     </dataValidation>
+    <dataValidation sqref="Q3:Q142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
+      <formula1>='下拉选项'!$J$2:$J$9</formula1>
+    </dataValidation>
     <dataValidation sqref="R3:R142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
-      <formula1>='下拉选项'!$J$2:$J$5</formula1>
+      <formula1>='下拉选项'!$K$2:$K$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="S3:S142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
+      <formula1>='下拉选项'!$L$2:$L$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="T3:T142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
+      <formula1>='下拉选项'!$M$2:$M$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="U3:U142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
+      <formula1>='下拉选项'!$N$2:$N$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="W3:W142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择，或留空。" type="list">
+      <formula1>='下拉选项'!$O$2:$O$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8421,7 +9240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -8434,6 +9253,11 @@
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8474,15 +9298,40 @@
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
+          <t>micro_example_applicability</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
           <t>leakage_label</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>preference_rank</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>overall_quality</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>would_show</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>needs_discussion</t>
+        </is>
+      </c>
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>review_status</t>
         </is>
@@ -8526,15 +9375,40 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>applicable｜适用：这条回复使用或应该使用微型例子</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>no_leakage｜无泄露：没有说穿当前关键桥</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>1｜同题中最好</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>5｜优秀：非常愿意给学生看</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>yes｜愿意：可以直接给学生看</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>high｜高：评分把握大</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>no｜不需要讨论</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>unlabeled｜未评</t>
         </is>
@@ -8578,15 +9452,40 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>not_applicable｜不适用：本轮不需要单独评价微型例子</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>minor_bridge_leakage｜轻微桥梁泄露：提示偏强但学生仍要推理</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>2｜同题中第二</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>4｜较好：可以给学生看，只有小问题</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>borderline｜勉强：需要人工改一下或有明显风险</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>medium｜中：基本确定，但可能有边界</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>yes｜需要讨论</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>labeled｜已评完</t>
         </is>
@@ -8628,41 +9527,89 @@
           <t>0｜差：例子和卡点关系弱，或直接替学生补完关键桥</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>major_bridge_leakage｜严重桥梁泄露：直接补完当前关键桥</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>3｜同题中第三</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>3｜可用：有帮助，但需要接受一些明显不足</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>no｜不愿意：不应给学生看</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>low｜低：证据不足或很难判断</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>needs_discussion｜不确定，需要讨论</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>N/A｜没有使用微型例子，无法单独评价</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>answer_leakage｜答案/代码泄露：给出完整题解、完整步骤或可提交代码</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>4｜同题中第四</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2｜勉强：问题较多，只能作为弱参考</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ai_prelim_reviewed｜AI 预评，待教练复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>5｜同题中第五</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1｜不可用：不建议给学生看</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>6｜同题中第六</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>7｜同题中第七</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="J9" t="inlineStr">
         <is>
           <t>tie｜并列/无法区分</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ai_prelim_reviewed｜AI 预评，待教练复核</t>
         </is>
       </c>
     </row>
@@ -8677,7 +9624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8783,24 +9730,84 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>泄露标签</t>
+          <t>微型例子是否适用</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>no_leakage=无泄露；minor=偏强但仍需推理；major=补完关键桥；answer=完整题解/步骤/代码泄露。</t>
+          <t>如果回复没有使用例子且本轮也不需要例子，选“不适用”，微型例子分数可留空。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>泄露标签</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>no_leakage=无泄露；minor=偏强但仍需推理；major=补完关键桥；answer=完整题解/步骤/代码泄露。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>同题回复排序</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>如果同一个 case 有多条回复，可填 1/2/3；只评单条时可留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>总体质量</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>1-5 的整体教练判断，用来表达细项平均分捕捉不到的整体可用性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>是否愿意给学生看</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>yes=可直接给学生；borderline=勉强；no=不建议给学生看。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>评分置信度</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>标低置信的样本后续应进入双标或裁决。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>是否需要讨论</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>用于标记边界样本、争议样本或需要第二位教练复核的样本。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document response review rubric v2
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/coach_response_review_workbook_fair_mini_study_20_20260511.zh.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/coach_response_review_workbook_fair_mini_study_20_20260511.zh.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +129,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9624,190 +9627,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>0-2 评分总原则</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>2=好，1=一般，0=差。评分对象是 AI 回复，不是学生。</t>
+          <t>维度</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>评分标准</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>例子</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>是否抓住卡点</t>
+          <t>0-2 评分总原则</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>看 AI 是否对准学生当前缺失的桥梁/卡点，而不是泛泛讲题解。</t>
+          <t>2=好；1=一般；0=差。评分对象是 AI 回复，不是学生。</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>如果回复不适用某个维度，先看适用性列或在备注里说明。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>是否贴合题目/对话</t>
+          <t>是否抓住卡点</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>看 AI 是否利用了题目、学生原话、近期对话或代码证据。</t>
+          <t>看 AI 是否对准学生当前缺失的桥梁/卡点，而不是泛泛讲题解。</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>学生问“状态怎么设”，高分回复应引导状态需要保留哪些信息；低分回复只说“DP 要找状态和转移”。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>帮助强度是否合适</t>
+          <t>是否贴合题目/对话</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>看 AI 是否给了合适脚手架；直接补答案/代码或只空泛追问都不好。</t>
+          <t>看 AI 是否利用了题目、学生原话、近期对话或代码证据。</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>lazy 场景中，围绕“区间加、区间求和、节点区间”展开，比泛泛说“lazy 是延迟更新”更贴合。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>是否控制关键桥泄露</t>
+          <t>帮助强度是否合适</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>看 AI 是否避免说穿学生本轮应该自己构造的状态、转移、check、公式、局部条件等。</t>
+          <t>看 AI 是否给了合适脚手架；直接补答案/代码或只空泛追问都不好。</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>学生只说“不会”，直接给完整转移是过强；只说“再想想”是过弱。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>下一步是否清楚</t>
+          <t>是否控制关键桥泄露</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>看学生读完后是否知道接下来要回答/尝试哪一步。</t>
+          <t>看 AI 是否避免说穿学生本轮应该自己构造的状态、转移、check、公式、局部条件等。</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>学生问 check(mid) true/false，直接给完整可行性条件和边界更新通常是关键桥泄露。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>是否保持单一焦点</t>
+          <t>下一步是否清楚</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>看回复是否围绕一个核心卡点，不同时抛出多个无关任务。</t>
+          <t>看学生读完后是否知道接下来要回答/尝试哪一步。</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>“先用一句话说 dp[j] 应记录什么”比“再思考状态和转移”更清楚。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>桥梁导向微型例子</t>
+          <t>是否保持单一焦点</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>如果用了例子，看它是否帮助学生提炼可迁移关系；只是让学生算一下/选一下但没有抽象方向，通常只能给 1。</t>
+          <t>看回复是否围绕一个核心卡点，不同时抛出多个无关任务。</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>学生卡在状态语义时，同时讲状态、转移、复杂度、代码模板，通常会让学生更乱。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>微型例子是否适用</t>
+          <t>桥梁导向微型例子</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>如果回复没有使用例子且本轮也不需要例子，选“不适用”，微型例子分数可留空。</t>
+          <t>如果用了例子，看它是否帮助学生提炼可迁移关系；只是让学生算一下/选一下但没有抽象方向，通常只能给 1。</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>lazy 例子里，只问“子节点有没有加 5”是局部任务；再追问“这说明 lazy 记录的是哪一层已生效、哪一层未下传”更桥梁导向。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>泄露标签</t>
+          <t>微型例子是否适用</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>no_leakage=无泄露；minor=偏强但仍需推理；major=补完关键桥；answer=完整题解/步骤/代码泄露。</t>
+          <t>如果回复没有使用例子且本轮也不需要例子，选“不适用”，微型例子分数可留空。</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>直接要完整代码的安全回复通常不需要微型例子，可选 not_applicable。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>同题回复排序</t>
+          <t>泄露标签</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>如果同一个 case 有多条回复，可填 1/2/3；只评单条时可留空。</t>
+          <t>no_leakage=无泄露；minor=偏强但仍需推理；major=补完关键桥；answer=完整题解/步骤/代码泄露。</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>直接给 dp 状态定义、完整转移式、check 条件，通常至少是 major_bridge_leakage。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>总体质量</t>
+          <t>同题回复排序</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>1-5 的整体教练判断，用来表达细项平均分捕捉不到的整体可用性。</t>
+          <t>同一个 case 有多条回复，可填 1-7；只评单条时可留空。</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>如果两个回复质量接近，可选 tie。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>是否愿意给学生看</t>
+          <t>总体质量</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>yes=可直接给学生；borderline=勉强；no=不建议给学生看。</t>
+          <t>1-5 的整体教练判断，用来表达细项平均分捕捉不到的整体可用性。</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>细项都一般但整体流畅可用，可给 3；很愿意给学生看可给 4 或 5。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>评分置信度</t>
+          <t>是否愿意给学生看</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>标低置信的样本后续应进入双标或裁决。</t>
+          <t>yes=可直接给学生；borderline=勉强；no=不建议给学生看。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>有明显泄题或答非所问时选 no；只需轻微人工改动时选 borderline。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>评分置信度</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>标低置信的样本后续应进入双标或裁决。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>题面信息不足、学生意图不清、多桥梁混合时可选 low 或 medium。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>是否需要讨论</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>用于标记边界样本、争议样本或需要第二位教练复核的样本。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>泄露程度介于 minor/major 之间，或不知道是否该给强提示时选 yes。</t>
         </is>
       </c>
     </row>

</xml_diff>